<commit_message>
Traffic Volume live update on map
</commit_message>
<xml_diff>
--- a/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
+++ b/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone\Project\Urban Traffic Sim\UrbanEcho\UrbanEcho\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B147A42-F81E-47F6-B7E6-E0F16D1A7896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0490FC71-86BF-4307-B946-513E38D0F8CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Title Page" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
   <si>
     <t>Report for:</t>
   </si>
@@ -96,9 +96,6 @@
     <t>{{item.TotalTimeSpent}}</t>
   </si>
   <si>
-    <t>{{item.NumberOfVehiclesEntered}}</t>
-  </si>
-  <si>
     <t>{{item.AverageWaitTime}}</t>
   </si>
   <si>
@@ -123,13 +120,13 @@
     <t>{{item.ToRoadName}}</t>
   </si>
   <si>
-    <t>{{item.NumberOfVehiclesExited}}</t>
-  </si>
-  <si>
     <t>RoadEdges Report</t>
   </si>
   <si>
     <t>Traffic Report</t>
+  </si>
+  <si>
+    <t>{{item.VehicleCount}}</t>
   </si>
 </sst>
 </file>
@@ -488,7 +485,7 @@
   <sheetData>
     <row r="4" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
       <c r="B4" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -511,7 +508,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
@@ -588,7 +585,7 @@
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
@@ -597,13 +594,13 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
         <v>22</v>
-      </c>
-      <c r="G8" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -659,10 +656,10 @@
         <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>13</v>
@@ -679,16 +676,16 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
         <v>20</v>
@@ -697,13 +694,13 @@
         <v>19</v>
       </c>
       <c r="G8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" t="s">
         <v>22</v>
-      </c>
-      <c r="I8" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made fixes to zoom to layer in the case where extents has NaN values. Updated report so that it includes a picutre of the map when exporting
</commit_message>
<xml_diff>
--- a/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
+++ b/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone\Project\Urban Traffic Sim\UrbanEcho\UrbanEcho\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0490FC71-86BF-4307-B946-513E38D0F8CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F3A43A-36F9-400B-A703-5D0600913464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Title Page" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>Report for:</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>{{item.VehicleCount}}</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Image Value=MapImage Scale=1.0&gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -511,6 +514,11 @@
         <v>29</v>
       </c>
     </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
     </row>

</xml_diff>

<commit_message>
made a fix where image was exported twice each call
</commit_message>
<xml_diff>
--- a/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
+++ b/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone\Project\Urban Traffic Sim\UrbanEcho\UrbanEcho\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F3A43A-36F9-400B-A703-5D0600913464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0467049E-92CB-4491-851D-A43669BEEEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7080" yWindow="3225" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Title Page" sheetId="3" r:id="rId1"/>

</xml_diff>

<commit_message>
changes for report (added a sheet that includes intersections and roads) made fix so vehicles do one update so path updates when they are created
</commit_message>
<xml_diff>
--- a/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
+++ b/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
@@ -8,30 +8,46 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone\Project\Urban Traffic Sim\UrbanEcho\UrbanEcho\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0467049E-92CB-4491-851D-A43669BEEEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFA31C5-B44B-424E-8693-EF47B3752990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7080" yWindow="3225" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Title Page" sheetId="3" r:id="rId1"/>
-    <sheet name="Intersections Report" sheetId="1" r:id="rId2"/>
-    <sheet name="Road Edges Report" sheetId="2" r:id="rId3"/>
+    <sheet name="Intersections With Road Report" sheetId="1" r:id="rId2"/>
+    <sheet name="Intersections Report" sheetId="4" r:id="rId3"/>
+    <sheet name="Road Report" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="Intersections">'Intersections Report'!$A$8:$G$9</definedName>
-    <definedName name="Roads">'Road Edges Report'!$A$8:$I$9</definedName>
+    <definedName name="Roads">'Road Report'!$A$8:$I$9</definedName>
+    <definedName name="TheReport" localSheetId="2">'Intersections Report'!$A$6:$J$10</definedName>
+    <definedName name="TheReport">'Intersections With Road Report'!$A$6:$M$13</definedName>
+    <definedName name="TheReport_Intersections" localSheetId="2">'Intersections Report'!$A$8:$J$9</definedName>
+    <definedName name="TheReport_Intersections">'Intersections With Road Report'!$A$7:$M$12</definedName>
+    <definedName name="TheReport_Intersections_Edges">'Intersections With Road Report'!$A$10:$M$11</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="37">
   <si>
     <t>Report for:</t>
   </si>
@@ -78,9 +94,6 @@
     <t>Road Edges Report</t>
   </si>
   <si>
-    <t>CREATED Date</t>
-  </si>
-  <si>
     <t>{{Date}}</t>
   </si>
   <si>
@@ -130,13 +143,28 @@
   </si>
   <si>
     <t>&lt;&lt;Image Value=MapImage Scale=1.0&gt;&gt;</t>
+  </si>
+  <si>
+    <t>Road Edges</t>
+  </si>
+  <si>
+    <t>{{item.BlankString}}</t>
+  </si>
+  <si>
+    <t>Intersections With Roads Report</t>
+  </si>
+  <si>
+    <t>Intersections With Road Details Report</t>
+  </si>
+  <si>
+    <t>CREATED Date {{Date}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,8 +187,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="16"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -169,17 +212,229 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="17">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -187,9 +442,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -197,13 +451,164 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -479,53 +884,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD7145E-817F-44B4-93B5-5CE06064E61C}">
-  <dimension ref="A4:B17"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
     <col min="2" max="2" width="143.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B4" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
-        <v>17</v>
+    <row r="1" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="51"/>
+      <c r="B2" s="52" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A3" s="51"/>
+      <c r="B3" s="51"/>
+    </row>
+    <row r="4" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A4" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="51"/>
+    </row>
+    <row r="5" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A5" s="51"/>
+      <c r="B5" s="51"/>
+    </row>
+    <row r="6" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A6" s="53" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A7" s="53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A8" s="54" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B15" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="3"/>
+      <c r="B10" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B13" location="'Intersections Report'!A1" display="Intersections Report" xr:uid="{2D620495-19D5-41A9-BD3F-499DCFE35A63}"/>
-    <hyperlink ref="B15" location="'Road Edges Report'!A1" display="RoadEdges Report" xr:uid="{C994D490-1F1E-4B98-941C-8EA20A43D2A3}"/>
+    <hyperlink ref="A7" location="'Intersections Report'!A1" display="Intersections Report" xr:uid="{2D620495-19D5-41A9-BD3F-499DCFE35A63}"/>
+    <hyperlink ref="A8" location="'Road Edges Report'!A1" display="RoadEdges Report" xr:uid="{C994D490-1F1E-4B98-941C-8EA20A43D2A3}"/>
+    <hyperlink ref="A6" location="'Intersections With Road Report'!A1" display="Intersections With Road Details Report" xr:uid="{01C6754A-7323-4EE3-B4F2-312E6A6023FE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -533,84 +951,180 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="B1:M13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="21.5703125" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="5" width="53.42578125" customWidth="1"/>
-    <col min="6" max="6" width="24.28515625" customWidth="1"/>
-    <col min="7" max="7" width="32.85546875" customWidth="1"/>
-    <col min="8" max="8" width="36.42578125" customWidth="1"/>
+    <col min="1" max="1" width="1.85546875" customWidth="1"/>
+    <col min="2" max="2" width="2.28515625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="2.85546875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="41.42578125" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" customWidth="1"/>
+    <col min="6" max="6" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" customWidth="1"/>
+    <col min="9" max="9" width="28.7109375" customWidth="1"/>
+    <col min="10" max="10" width="25.5703125" customWidth="1"/>
+    <col min="11" max="11" width="19" customWidth="1"/>
+    <col min="12" max="12" width="16.140625" customWidth="1"/>
+    <col min="13" max="13" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="4:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="22"/>
+    </row>
+    <row r="8" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="31" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="E8" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="L8" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" s="34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="49" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="L9" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="M9" s="20" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="10" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D10" s="49"/>
+      <c r="E10" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="K10" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="L10" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="M10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="G8" t="s">
-        <v>22</v>
-      </c>
-    </row>
+    </row>
+    <row r="11" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D11" s="50"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
+      <c r="M11" s="30"/>
+    </row>
+    <row r="12" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -618,18 +1132,127 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8D7773-B908-4AE1-8F78-AFB1C85B2E50}">
-  <dimension ref="A1:I8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6181B37F-6738-45A7-AF37-53A17D9D947A}">
+  <dimension ref="B1:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="3" width="22.140625" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="39.5703125" customWidth="1"/>
-    <col min="6" max="6" width="30.28515625" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" customWidth="1"/>
-    <col min="8" max="8" width="39.140625" customWidth="1"/>
-    <col min="9" max="9" width="37.28515625" customWidth="1"/>
+    <col min="1" max="1" width="1.85546875" style="35" customWidth="1"/>
+    <col min="2" max="2" width="2.28515625" style="35" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="2.85546875" style="35" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="41.42578125" style="35" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" style="35" customWidth="1"/>
+    <col min="6" max="6" width="27.5703125" style="35" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" style="35" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" style="35" customWidth="1"/>
+    <col min="9" max="9" width="28.7109375" style="35" customWidth="1"/>
+    <col min="10" max="10" width="25.5703125" style="35" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="35"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="D1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="35" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="D3" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="D5" s="35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="4:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="4:10" s="36" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="44" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="I7" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="46" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="4:10" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="47" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="4:10" s="36" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="40"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="43"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="48"/>
+    </row>
+    <row r="10" spans="4:10" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="4:10" s="36" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8D7773-B908-4AE1-8F78-AFB1C85B2E50}">
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -637,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -645,7 +1268,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -653,65 +1276,82 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:9" s="5" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="C8" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="D8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="I8" t="s">
-        <v>22</v>
-      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="10"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="13"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Made changes so report exports on a different task Made smaller template so it takes less time Added change so if one report is being created it will just show a message saying other report already in progress
</commit_message>
<xml_diff>
--- a/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
+++ b/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone\Project\Urban Traffic Sim\UrbanEcho\UrbanEcho\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFA31C5-B44B-424E-8693-EF47B3752990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAE2827-4889-431D-B866-CAC63EEBE40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,9 +142,6 @@
     <t>{{item.VehicleCount}}</t>
   </si>
   <si>
-    <t>&lt;&lt;Image Value=MapImage Scale=1.0&gt;&gt;</t>
-  </si>
-  <si>
     <t>Road Edges</t>
   </si>
   <si>
@@ -158,6 +155,9 @@
   </si>
   <si>
     <t>CREATED Date {{Date}}</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Image Value=MapImage Scale=2.0&gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -908,7 +908,7 @@
     </row>
     <row r="4" spans="1:2" ht="21" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="51"/>
     </row>
@@ -918,7 +918,7 @@
     </row>
     <row r="6" spans="1:2" ht="21" x14ac:dyDescent="0.35">
       <c r="A6" s="53" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="21" x14ac:dyDescent="0.35">
@@ -933,7 +933,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -987,7 +987,7 @@
     </row>
     <row r="5" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="4:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -1040,18 +1040,18 @@
         <v>21</v>
       </c>
       <c r="K8" s="33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L8" s="33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M8" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D9" s="49" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Removed conditional formatting in report so it generates faster
</commit_message>
<xml_diff>
--- a/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
+++ b/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone\Project\Urban Traffic Sim\UrbanEcho\UrbanEcho\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAE2827-4889-431D-B866-CAC63EEBE40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153BD9E3-152C-4B6E-A06C-BB7DE1F66D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="Road Report" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="Roads">'Road Report'!$A$8:$I$9</definedName>
+    <definedName name="Roads">'Road Report'!$A$8:$J$9</definedName>
     <definedName name="TheReport" localSheetId="2">'Intersections Report'!$A$6:$J$10</definedName>
     <definedName name="TheReport">'Intersections With Road Report'!$A$6:$M$13</definedName>
     <definedName name="TheReport_Intersections" localSheetId="2">'Intersections Report'!$A$8:$J$9</definedName>
@@ -235,102 +235,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -437,52 +347,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -491,40 +393,40 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -533,14 +435,42 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -549,66 +479,61 @@
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -887,57 +812,58 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="143.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="21" customWidth="1"/>
+    <col min="2" max="2" width="143.5703125" style="21" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="27" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="51"/>
-      <c r="B2" s="52" t="s">
+      <c r="A2" s="28"/>
+      <c r="B2" s="29" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="51"/>
-      <c r="B3" s="51"/>
+      <c r="A3" s="28"/>
+      <c r="B3" s="28"/>
     </row>
     <row r="4" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="51"/>
+      <c r="B4" s="28"/>
     </row>
     <row r="5" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A5" s="51"/>
-      <c r="B5" s="51"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
     </row>
     <row r="6" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="30" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="30" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A8" s="54" t="s">
+      <c r="A8" s="31" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="32" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
+      <c r="B10" s="33"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -991,140 +917,140 @@
       </c>
     </row>
     <row r="6" spans="4:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7" s="16" t="s">
+    <row r="7" spans="4:13" s="1" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="17" t="s">
+      <c r="H7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="I7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="22"/>
-    </row>
-    <row r="8" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D8" s="31" t="s">
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="8"/>
+    </row>
+    <row r="8" spans="4:13" s="1" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="33" t="s">
+      <c r="F8" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="G8" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="33" t="s">
+      <c r="H8" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="33" t="s">
+      <c r="I8" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="33" t="s">
+      <c r="J8" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="33" t="s">
+      <c r="K8" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="L8" s="33" t="s">
+      <c r="L8" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="M8" s="34" t="s">
+      <c r="M8" s="20" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D9" s="49" t="s">
+    <row r="9" spans="4:13" s="1" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="19" t="s">
+      <c r="J9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="19" t="s">
+      <c r="K9" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="L9" s="19" t="s">
+      <c r="L9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="M9" s="20" t="s">
+      <c r="M9" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D10" s="49"/>
-      <c r="E10" s="23" t="s">
+    <row r="10" spans="4:13" s="1" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D10" s="25"/>
+      <c r="E10" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="23" t="s">
+      <c r="G10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="I10" s="25" t="s">
+      <c r="I10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="25" t="s">
+      <c r="J10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="K10" s="25" t="s">
+      <c r="K10" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="L10" s="25" t="s">
+      <c r="L10" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="M10" s="26" t="s">
+      <c r="M10" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D11" s="50"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="29"/>
-      <c r="L11" s="29"/>
-      <c r="M11" s="30"/>
-    </row>
-    <row r="12" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="4:13" s="4" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="4:13" s="1" customFormat="1" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D11" s="26"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="16"/>
+    </row>
+    <row r="12" spans="4:13" s="1" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="4:13" s="1" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -1136,104 +1062,99 @@
   <dimension ref="B1:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" style="35" customWidth="1"/>
-    <col min="2" max="2" width="2.28515625" style="35" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="2.85546875" style="35" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="41.42578125" style="35" customWidth="1"/>
-    <col min="5" max="5" width="24.5703125" style="35" customWidth="1"/>
-    <col min="6" max="6" width="27.5703125" style="35" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.5703125" style="35" customWidth="1"/>
-    <col min="8" max="8" width="24.42578125" style="35" customWidth="1"/>
-    <col min="9" max="9" width="28.7109375" style="35" customWidth="1"/>
-    <col min="10" max="10" width="25.5703125" style="35" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="35"/>
+    <col min="1" max="1" width="1.85546875" style="21" customWidth="1"/>
+    <col min="2" max="2" width="2.28515625" style="21" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="2.85546875" style="21" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="41.42578125" style="21" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" style="21" customWidth="1"/>
+    <col min="6" max="6" width="27.5703125" style="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" style="21" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" style="21" customWidth="1"/>
+    <col min="9" max="9" width="28.7109375" style="21" customWidth="1"/>
+    <col min="10" max="10" width="25.5703125" style="21" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="21" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="21" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="21" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="4:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="4:10" s="36" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7" s="44" t="s">
+    <row r="7" spans="4:10" s="34" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="45" t="s">
+      <c r="E7" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="45" t="s">
+      <c r="F7" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="45" t="s">
+      <c r="H7" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="I7" s="45" t="s">
+      <c r="I7" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="46" t="s">
+      <c r="J7" s="24" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="4:10" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D8" s="37" t="s">
+    <row r="8" spans="4:10" s="34" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="38" t="s">
+      <c r="E8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="39" t="s">
+      <c r="G8" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="39" t="s">
+      <c r="I8" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="47" t="s">
+      <c r="J8" s="38" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="4:10" s="36" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="42"/>
-      <c r="H9" s="43"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="48"/>
-    </row>
-    <row r="10" spans="4:10" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="4:10" s="36" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="4:10" s="34" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="39"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="43"/>
+    </row>
+    <row r="10" spans="4:10" s="34" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="4:10" s="34" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -1241,116 +1162,114 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8D7773-B908-4AE1-8F78-AFB1C85B2E50}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="B1:J9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.42578125" style="21" customWidth="1"/>
+    <col min="2" max="2" width="33" style="21" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" style="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23" style="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" style="21" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" style="21" customWidth="1"/>
+    <col min="9" max="9" width="24.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22" style="21" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="21" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="21" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="21" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="5" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+    <row r="6" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:10" s="44" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B7" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="C7" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="E7" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="F7" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="G7" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="H7" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="I7" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="J7" s="24" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="C8" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="G8" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="H8" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="I8" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="J8" s="54" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="13"/>
+    <row r="9" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="45"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="47"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="49"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Made a change so picture of map displays volume correct on report, fixed a problem that caused report from generating because map was being updated during tracking, made tracking more smooth, made update so pin for tracking is centered on vehicle
</commit_message>
<xml_diff>
--- a/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
+++ b/UrbanEcho/UrbanEcho/Resources/Templates/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone\Project\Urban Traffic Sim\UrbanEcho\UrbanEcho\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153BD9E3-152C-4B6E-A06C-BB7DE1F66D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBE2B2B-493A-468F-AC1C-B47329CC92C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -157,7 +157,7 @@
     <t>CREATED Date {{Date}}</t>
   </si>
   <si>
-    <t>&lt;&lt;Image Value=MapImage Scale=2.0&gt;&gt;</t>
+    <t>&lt;&lt;Image Value=MapImage Scale=1.0&gt;&gt;</t>
   </si>
 </sst>
 </file>

</xml_diff>